<commit_message>
chore(data-release): publish site data 2026-10-30 15:50:06 UTC
</commit_message>
<xml_diff>
--- a/countries/at/1990-1994.xlsx
+++ b/countries/at/1990-1994.xlsx
@@ -765,6 +765,11 @@
       <c r="O2" t="n">
         <v>103</v>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
           <t>SER_AT_ECDC_AIDS_ANNUAL</t>
@@ -782,7 +787,12 @@
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
@@ -792,6 +802,11 @@
       </c>
       <c r="AT2" t="n">
         <v>1</v>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV2" t="inlineStr">
         <is>
@@ -857,7 +872,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -872,17 +887,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>D162</t>
+          <t>D005</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>HIV infection</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>人类免疫缺乏病毒感染</t>
+          <t>艾滋病</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -901,14 +916,39 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>247</v>
+        <v>103</v>
       </c>
       <c r="O3" t="n">
-        <v>247</v>
+        <v>103</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -916,6 +956,64 @@
           <t>annual</t>
         </is>
       </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN3" t="b">
+        <v>1</v>
+      </c>
       <c r="AO3" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -923,16 +1021,26 @@
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
         </is>
       </c>
       <c r="AT3" t="n">
         <v>1</v>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV3" t="inlineStr">
         <is>
@@ -1013,17 +1121,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>D005</t>
+          <t>D162</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>HIV infection</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>艾滋病</t>
+          <t>人类免疫缺乏病毒感染</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1033,23 +1141,28 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1991-01-01</t>
+          <t>1990-01-01</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>1991-01</t>
+          <t>1990-01</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>123</v>
+        <v>247</v>
       </c>
       <c r="O4" t="n">
-        <v>123</v>
+        <v>247</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -1064,16 +1177,26 @@
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
         </is>
       </c>
       <c r="AT4" t="n">
         <v>1</v>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV4" t="inlineStr">
         <is>
@@ -1139,7 +1262,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1174,30 +1297,113 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1991-01-01</t>
+          <t>1990-01-01</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1991-01</t>
+          <t>1990-01</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>226</v>
+        <v>247</v>
       </c>
       <c r="O5" t="n">
-        <v>226</v>
+        <v>247</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
           <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
       <c r="AA5" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN5" t="b">
+        <v>1</v>
+      </c>
       <c r="AO5" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -1205,7 +1411,12 @@
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
@@ -1215,6 +1426,11 @@
       </c>
       <c r="AT5" t="n">
         <v>1</v>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV5" t="inlineStr">
         <is>
@@ -1315,19 +1531,24 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1992-01-01</t>
+          <t>1991-01-01</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>1992-01</t>
+          <t>1991-01</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>150</v>
+        <v>123</v>
       </c>
       <c r="O6" t="n">
-        <v>150</v>
+        <v>123</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1346,7 +1567,12 @@
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
@@ -1356,6 +1582,11 @@
       </c>
       <c r="AT6" t="n">
         <v>1</v>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV6" t="inlineStr">
         <is>
@@ -1421,7 +1652,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1436,17 +1667,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>D162</t>
+          <t>D005</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>HIV infection</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>人类免疫缺乏病毒感染</t>
+          <t>艾滋病</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1456,23 +1687,48 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1992-01-01</t>
+          <t>1991-01-01</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>1992-01</t>
+          <t>1991-01</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>300</v>
+        <v>123</v>
       </c>
       <c r="O7" t="n">
-        <v>300</v>
+        <v>123</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1480,6 +1736,64 @@
           <t>annual</t>
         </is>
       </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN7" t="b">
+        <v>1</v>
+      </c>
       <c r="AO7" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -1487,16 +1801,26 @@
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
         </is>
       </c>
       <c r="AT7" t="n">
         <v>1</v>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV7" t="inlineStr">
         <is>
@@ -1577,17 +1901,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>D005</t>
+          <t>D162</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>AIDS</t>
+          <t>HIV infection</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>艾滋病</t>
+          <t>人类免疫缺乏病毒感染</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1597,23 +1921,28 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1993-01-01</t>
+          <t>1991-01-01</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>1993-01</t>
+          <t>1991-01</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>155</v>
+        <v>226</v>
       </c>
       <c r="O8" t="n">
-        <v>155</v>
+        <v>226</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -1628,16 +1957,26 @@
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
         </is>
       </c>
       <c r="AT8" t="n">
         <v>1</v>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV8" t="inlineStr">
         <is>
@@ -1703,7 +2042,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1738,30 +2077,113 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1993-01-01</t>
+          <t>1991-01-01</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>1993-01</t>
+          <t>1991-01</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>259</v>
+        <v>226</v>
       </c>
       <c r="O9" t="n">
-        <v>259</v>
+        <v>226</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
           <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
         </is>
       </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
       <c r="AA9" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN9" t="b">
+        <v>1</v>
+      </c>
       <c r="AO9" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -1769,7 +2191,12 @@
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
@@ -1779,6 +2206,11 @@
       </c>
       <c r="AT9" t="n">
         <v>1</v>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV9" t="inlineStr">
         <is>
@@ -1879,19 +2311,24 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1994-01-01</t>
+          <t>1992-01-01</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>1994-01</t>
+          <t>1992-01</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="O10" t="n">
-        <v>154</v>
+        <v>150</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1910,7 +2347,12 @@
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
@@ -1920,6 +2362,11 @@
       </c>
       <c r="AT10" t="n">
         <v>1</v>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
       </c>
       <c r="AV10" t="inlineStr">
         <is>
@@ -1985,7 +2432,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2000,17 +2447,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>D162</t>
+          <t>D005</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>HIV infection</t>
+          <t>AIDS</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>人类免疫缺乏病毒感染</t>
+          <t>艾滋病</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2020,23 +2467,48 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1994-01-01</t>
+          <t>1992-01-01</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>1994-01</t>
+          <t>1992-01</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>223</v>
+        <v>150</v>
       </c>
       <c r="O11" t="n">
-        <v>223</v>
+        <v>150</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
@@ -2044,6 +2516,64 @@
           <t>annual</t>
         </is>
       </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN11" t="b">
+        <v>1</v>
+      </c>
       <c r="AO11" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -2051,17 +2581,27 @@
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
         </is>
       </c>
       <c r="AT11" t="n">
         <v>1</v>
       </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
       <c r="AV11" t="inlineStr">
         <is>
           <t>ages_radar</t>
@@ -2098,6 +2638,1956 @@
         </is>
       </c>
       <c r="BC11" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>D162</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>人类免疫缺乏病毒感染</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1992-01-01</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>1992-01</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>300</v>
+      </c>
+      <c r="O12" t="n">
+        <v>300</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>D162</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>人类免疫缺乏病毒感染</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1992-01-01</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>1992-01</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>300</v>
+      </c>
+      <c r="O13" t="n">
+        <v>300</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>D005</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>艾滋病</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1993-01-01</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>1993-01</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>155</v>
+      </c>
+      <c r="O14" t="n">
+        <v>155</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>D005</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>艾滋病</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>1993-01-01</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>1993-01</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>155</v>
+      </c>
+      <c r="O15" t="n">
+        <v>155</v>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN15" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>D162</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>人类免疫缺乏病毒感染</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1993-01-01</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>1993-01</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>259</v>
+      </c>
+      <c r="O16" t="n">
+        <v>259</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>D162</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>人类免疫缺乏病毒感染</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>1993-01-01</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>1993-01</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>259</v>
+      </c>
+      <c r="O17" t="n">
+        <v>259</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN17" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC17" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>D005</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>艾滋病</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1994-01-01</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>1994-01</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>154</v>
+      </c>
+      <c r="O18" t="n">
+        <v>154</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>D005</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>艾滋病</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1994-01-01</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>1994-01</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>154</v>
+      </c>
+      <c r="O19" t="n">
+        <v>154</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>AIDS</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_AIDS_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC19" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>D162</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>人类免疫缺乏病毒感染</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>1994-01-01</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>1994-01</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>223</v>
+      </c>
+      <c r="O20" t="n">
+        <v>223</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>missing_population</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC20" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>at</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>D162</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>人类免疫缺乏病毒感染</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>1994-01-01</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>1994-01</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>223</v>
+      </c>
+      <c r="O21" t="n">
+        <v>223</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>SRC_AT_ECDC_ATLAS</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>HIV infection</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>ecdc_member_state_reported_aggregate_surveillance</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>country:AT:national</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>ECDC_CURRENT_GENERAL_ANNUAL_2026_08</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>Austria annual Member-State reported aggregate cases from the public ECDC Surveillance Atlas; published zeroes are explicit, absent topic/year cells remain unknown, and combined populations are emitted only when every reviewed component is present. Data provided by ECDC based on data reported by EU/EEA Member States.</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="AN21" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>SER_AT_ECDC_HIV_INFECTION_ANNUAL</t>
+        </is>
+      </c>
+      <c r="AT21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>official_monthly_csv</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>ages_radar</t>
+        </is>
+      </c>
+      <c r="BA21" t="inlineStr">
+        <is>
+          <t>Austria AGES Radar for Infectious Diseases</t>
+        </is>
+      </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>https://www.ages.at/en/human/disease/ages-radar-for-infectious-diseases</t>
+        </is>
+      </c>
+      <c r="BC21" t="inlineStr">
         <is>
           <t>official_monthly_csv</t>
         </is>
@@ -2229,7 +4719,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
@@ -2249,7 +4739,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -2259,7 +4749,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">

</xml_diff>